<commit_message>
Numbers audit: every deck figure re-verified against logs, reports, sources and live prices
- BOM re-quoted 9 Oct 2026: Rs 33,945 (Rs 3,945 over grant); Pi 5, Tang Nano 9K, TF-Luna out of stock
- Runtime unified to 3.1 / 4.3 / 7.2 h (event-triggered assumes ~50 % AI duty); one component list for sheet + analysis
- Latency: 136 ns on waveform vs <= 214 ns conservative testbench bound, explained
- Citations checked: Manduchi survey stats (307 resp., 13 % / 7 % monthly), OrCam US$4,250, SmartCane 2016
- Detection chart: AP50 per class with n, large-object recall only where >= 5 samples; e2e label clarified
- FEA convergence wording (<= 3 %), v2 FoS 8.7 (all runs >= 8.6)
- Evidence added: 44 mm CAD clash re-run (182.26 mm3, 170.6 HDMI), KiCad DRC/ERC/parity re-run, OCR word-order re-check (25.78 -> 1.91 %)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/design/bom/VisionAid_BOM_Power.xlsx
+++ b/design/bom/VisionAid_BOM_Power.xlsx
@@ -455,7 +455,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VisionAid prototype BOM (Stage 2 design). Quote = listing checked 8 Oct 2026; Estimate = verify before ordering.</t>
+          <t>VisionAid prototype BOM (Stage 2 design). Quote = live listing checked 9 Oct 2026; Estimate = verify before ordering.</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>12000</v>
+        <v>14500</v>
       </c>
       <c r="F3">
         <f>D3*E3</f>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>KSP Electronics listing (in stock); guides quote 5.5-7.5k</t>
+          <t>kspelectronics.in INR 14,500 incl. GST (out of stock, 9 Oct); electronifyindia.com INR 12,600 (sold out)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2-4 days</t>
+          <t>stock-dependent</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>2149</v>
+        <v>2999</v>
       </c>
       <c r="F6">
         <f>D6*E6</f>
@@ -685,7 +685,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Probots.co.in (incl. GST)</t>
+          <t>probots.co.in INR 2,999 incl. GST (out of stock, 9 Oct)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1-3 days</t>
+          <t>stock-dependent</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>3250</v>
+        <v>3158</v>
       </c>
       <c r="F7">
         <f>D7*E7</f>
@@ -732,7 +732,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Thingbits.in</t>
+          <t>thingbits.in INR 3,157.68 incl. GST (in stock, 9 Oct)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Probots.co.in (incl. GST)</t>
+          <t>probots.co.in INR 2,118 incl. GST (out of stock, 9 Oct)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>1-3 days</t>
+          <t>stock-dependent</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PETG 1 kg (enclosure ~140 g solid volume)</t>
+          <t>PETG 1 kg (enclosure ~156 g if printed solid: 123 cm3 x 1.27 g/cm3)</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>At the highest Pi 5 quote (INR 12,000) the build is ~INR 700 over the grant. At the INR 5,500-7,500 distributor price it is ~INR 24-26k. Rule: buy the Pi 5 4 GB only at &lt;= INR 9,000, otherwise a Pi 4 4 GB (lower AI frame rate, same design).</t>
+          <t>Everything except the Pi 5 board costs INR 19,445, so the Pi 5 4 GB must cost &lt;= INR 10,555 to stay inside the INR 30,000 grant. On 9 Oct 2026 the checked listings were INR 12,600-14,500 and out of stock, i.e. INR 2,045-3,945 over. Rule: re-quote at order time; if no Pi 5 4 GB &lt;= INR 10,555, cover the gap from team funds or move to a cheaper board (re-quote and re-test in Stage 3).</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1587,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Raspberry Pi 5 (camera + YOLO running)</t>
+          <t>Raspberry Pi 5, event-triggered AI</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1599,11 +1599,11 @@
         <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Assumption - to be measured (Stage 3, USB-C meter)</t>
+          <t>Cited 3.0 W idle / 8.8 W full load (raspberry.tips 2026), AI busy ~50 % (assumption) -&gt; 5.9 W; measure in Stage 3</t>
         </is>
       </c>
     </row>

</xml_diff>